<commit_message>
Correction du KeyError Taux_Obs et nettoyage Unicode pour le PDF
</commit_message>
<xml_diff>
--- a/outputs/Reporting_VaR.xlsx
+++ b/outputs/Reporting_VaR.xlsx
@@ -22,10 +22,10 @@
     <t>Exceptions</t>
   </si>
   <si>
-    <t>Taux_Obs</t>
-  </si>
-  <si>
-    <t>P_value_Kupiec</t>
+    <t>Taux Obs (%)</t>
+  </si>
+  <si>
+    <t>P_value</t>
   </si>
   <si>
     <t>Statut</t>
@@ -52,7 +52,7 @@
     <t>TVE-Garch</t>
   </si>
   <si>
-    <t>Valide</t>
+    <t>✅ Valide</t>
   </si>
 </sst>
 </file>
@@ -435,13 +435,13 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>0.6571</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
@@ -452,13 +452,13 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C3">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>0.1632</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
@@ -469,13 +469,13 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>0.1632</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
@@ -486,13 +486,13 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>0.8853</v>
+        <v>1</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -503,13 +503,13 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>0.4529</v>
+        <v>1</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -520,13 +520,13 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>0.4529</v>
+        <v>1</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -537,13 +537,13 @@
         <v>11</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="D8">
-        <v>0.8853</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>

</xml_diff>